<commit_message>
Clinical or Microbiological field added in TBDetails
</commit_message>
<xml_diff>
--- a/Patient_ReportDead.xlsx
+++ b/Patient_ReportDead.xlsx
@@ -40,30 +40,20 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <sz val="14.0"/>
       <b val="true"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="darkGray"/>
     </fill>
-    <fill>
-      <patternFill patternType="none">
-        <fgColor indexed="48"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor indexed="48"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="5">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -71,34 +61,13 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <bottom style="thin"/>
-    </border>
-    <border>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
-    <border>
-      <left style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="true" applyAlignment="true" applyFill="true" applyBorder="true">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyAlignment="true" applyBorder="true">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -110,8 +79,8 @@
   <dimension ref="A1:B3"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="19.53125" customWidth="true"/>
-    <col min="2" max="2" width="11.71875" customWidth="true"/>
+    <col min="1" max="1" width="27.34375" customWidth="true"/>
+    <col min="2" max="2" width="27.34375" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -123,19 +92,19 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="s" s="2">
+      <c r="A2" t="s" s="0">
         <v>2</v>
       </c>
-      <c r="B2" t="n" s="2">
-        <v>13.0</v>
+      <c r="B2" t="n" s="0">
+        <v>0.0</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="s" s="2">
+      <c r="A3" t="s" s="0">
         <v>3</v>
       </c>
-      <c r="B3" t="n" s="2">
-        <v>1.0</v>
+      <c r="B3" t="n" s="0">
+        <v>0.0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>